<commit_message>
feat: implement enhanced security and compliance controls
- Add immediate token/session revocation for user termination
- Enforce PKCE flow and secure server-side auth
- Remove hardcoded credentials and email-based RBAC
- Update compliance audit report with new security mitigations
- Add comprehensive automation execution audit logging
</commit_message>
<xml_diff>
--- a/docs/HIPAA_ISO27001_Credentialing_Compliance_Audit_Report.xlsx
+++ b/docs/HIPAA_ISO27001_Credentialing_Compliance_Audit_Report.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="468">
   <si>
     <t>PROFICIO HEALTHCARE CREDENTIALING PLATFORM</t>
   </si>
@@ -29,7 +29,7 @@
     <t>Audit Assessment Date:</t>
   </si>
   <si>
-    <t>2026-09-15 09:01:24 UTC</t>
+    <t>2026-09-15 13:21:06 UTC</t>
   </si>
   <si>
     <t>Audit Scope:</t>
@@ -476,6 +476,141 @@
     <t>Simulated Clinical Coordinator switching to Admin tab; automatically redirected to authorized dashboard.</t>
   </si>
   <si>
+    <t>SEC-HASH-01</t>
+  </si>
+  <si>
+    <t>HIPAA §164.312(a)(1) &amp; ISO A.8.5</t>
+  </si>
+  <si>
+    <t>Plaintext seed credentials stored in code; potential credential exposure during audit inspection.</t>
+  </si>
+  <si>
+    <t>Removed all plaintext credentials, implemented SHA-256 passwordHash mapping and zero-knowledge verification.</t>
+  </si>
+  <si>
+    <t>src/data/initialData.ts &amp; CredentialingContext.tsx</t>
+  </si>
+  <si>
+    <t>Verified seed account objects contain zero password strings; authenticated using cryptographic hash comparator.</t>
+  </si>
+  <si>
+    <t>SEC-RBAC-02</t>
+  </si>
+  <si>
+    <t>Hardcoded administrative emails (admin@example.com) granted superadmin privileges.</t>
+  </si>
+  <si>
+    <t>Refactored isSuperAdmin to enforce dynamic accessLevel, permissions, and systemRole attributes.</t>
+  </si>
+  <si>
+    <t>src/utils/rbac.ts, CredentialingContext.tsx, authGate.ts</t>
+  </si>
+  <si>
+    <t>Verified accounts evaluated strictly by role entitlements; all hardcoded email dependencies eradicated.</t>
+  </si>
+  <si>
+    <t>SEC-REVOKE-01</t>
+  </si>
+  <si>
+    <t>HIPAA §164.308(a)(3)(ii)(C)</t>
+  </si>
+  <si>
+    <t>Missing immediate token and session revocation when accounts are deactivated or terminated.</t>
+  </si>
+  <si>
+    <t>Engineered revokeAllTokens() and invalidateAllSessions() triggered synchronously on user deactivation.</t>
+  </si>
+  <si>
+    <t>src/lib/supabase.ts, NewUserView.tsx, server/authGate.ts</t>
+  </si>
+  <si>
+    <t>Deactivated test account; verified active tokens purged, session cleared, and audit record generated.</t>
+  </si>
+  <si>
+    <t>SEC-MFA-01</t>
+  </si>
+  <si>
+    <t>Auth configuration lacked Multi-Factor Authentication (MFA) verification enforcement.</t>
+  </si>
+  <si>
+    <t>Upgraded client &amp; server auth to PKCE flow and added checkMfaStatus() verification helper.</t>
+  </si>
+  <si>
+    <t>src/lib/supabase.ts &amp; server/authGate.ts</t>
+  </si>
+  <si>
+    <t>Verified PKCE auth initialization and MFA authenticator assurance level validation.</t>
+  </si>
+  <si>
+    <t>SEC-BREACH-01</t>
+  </si>
+  <si>
+    <t>HIPAA §164.308(a)(6)(ii)</t>
+  </si>
+  <si>
+    <t>Missing automated breach notification and security incident tracking mechanism.</t>
+  </si>
+  <si>
+    <t>Implemented reportSecurityIncident() logging security alerts on unauthorized access attempts.</t>
+  </si>
+  <si>
+    <t>server/authGate.ts</t>
+  </si>
+  <si>
+    <t>Simulated unauthorized OAuth login; verified security_incidents audit trail entry logged.</t>
+  </si>
+  <si>
+    <t>SEC-MIN-02</t>
+  </si>
+  <si>
+    <t>HIPAA §164.502(b)</t>
+  </si>
+  <si>
+    <t>SELECT * database queries on PHI tables violated the Minimum Necessary principle.</t>
+  </si>
+  <si>
+    <t>Restricted all table queries to explicit column projections (users, providers, records, entities).</t>
+  </si>
+  <si>
+    <t>Inspected database query payloads; verified only authorized columns retrieved over the wire.</t>
+  </si>
+  <si>
+    <t>SEC-ALERT-01</t>
+  </si>
+  <si>
+    <t>Accessibility &amp; Resiliency</t>
+  </si>
+  <si>
+    <t>Synchronous window.alert calls in automation dashboard could freeze thread in iframe.</t>
+  </si>
+  <si>
+    <t>Replaced window.alert with non-blocking dismissible error banner and state handler.</t>
+  </si>
+  <si>
+    <t>src/components/automations/AutomationDashboardView.tsx</t>
+  </si>
+  <si>
+    <t>Triggered automation error condition; verified non-blocking UI alert banner displayed without freezing.</t>
+  </si>
+  <si>
+    <t>SEC-AUDIT-02</t>
+  </si>
+  <si>
+    <t>ISO 27001:2022 A.12.4.1</t>
+  </si>
+  <si>
+    <t>Automated cron executions and document deletions lacked full audit trail persistence.</t>
+  </si>
+  <si>
+    <t>Added audit_logs insertion in recordExecution() and deleteDocument() routines.</t>
+  </si>
+  <si>
+    <t>server/automationEngine.ts &amp; src/lib/supabase.ts</t>
+  </si>
+  <si>
+    <t>Executed automation cycle and document deletion; verified audit_logs records created in database.</t>
+  </si>
+  <si>
     <t>Standard §</t>
   </si>
   <si>
@@ -1092,6 +1227,60 @@
   </si>
   <si>
     <t>Completely removed all quick-fill buttons and dev shortcut UI elements</t>
+  </si>
+  <si>
+    <t>src/data/initialData.ts</t>
+  </si>
+  <si>
+    <t>Data Model &amp; Seeds</t>
+  </si>
+  <si>
+    <t>Plaintext seed passwords exposed in source code repository</t>
+  </si>
+  <si>
+    <t>Replaced all plaintext passwords with zero-knowledge SHA-256 passwordHash mapping</t>
+  </si>
+  <si>
+    <t>Server Auth &amp; SSO</t>
+  </si>
+  <si>
+    <t>Hardcoded superadmin email bypass and unlogged unauthorized access</t>
+  </si>
+  <si>
+    <t>Implemented role-based verification, automated breach incident reporting, token revocation</t>
+  </si>
+  <si>
+    <t>src/components/admin/NewUserView.tsx</t>
+  </si>
+  <si>
+    <t>User Administration</t>
+  </si>
+  <si>
+    <t>User deletion did not immediately revoke active sessions/tokens</t>
+  </si>
+  <si>
+    <t>Integrated revokeAllTokens() and invalidateAllSessions() upon account deletion</t>
+  </si>
+  <si>
+    <t>Resiliency &amp; UI</t>
+  </si>
+  <si>
+    <t>Synchronous window.alert calls in automation dashboard</t>
+  </si>
+  <si>
+    <t>Replaced with non-blocking responsive inline error alert state</t>
+  </si>
+  <si>
+    <t>server/automationEngine.ts</t>
+  </si>
+  <si>
+    <t>Automation Engine</t>
+  </si>
+  <si>
+    <t>Automated job cycles executed without ISO 27001 event audit logging</t>
+  </si>
+  <si>
+    <t>Integrated ISO 27001 A.12.4.1 immutable audit trail logging on job lifecycle</t>
   </si>
   <si>
     <t>Phase</t>
@@ -2362,7 +2551,7 @@
   <sheetPr>
     <tabColor rgb="FF059669"/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2683,6 +2872,214 @@
         <v>90</v>
       </c>
       <c r="H12" s="21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="G13" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H13" s="21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>162</v>
+      </c>
+      <c r="G14" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H14" s="21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="21" t="s">
+        <v>163</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="G15" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H15" s="21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="21" t="s">
+        <v>169</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>171</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H16" s="21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="21" t="s">
+        <v>174</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="D17" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>179</v>
+      </c>
+      <c r="G17" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H17" s="21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="21" t="s">
+        <v>180</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>181</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>182</v>
+      </c>
+      <c r="D18" s="22" t="s">
+        <v>183</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="F18" s="22" t="s">
+        <v>184</v>
+      </c>
+      <c r="G18" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H18" s="21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>188</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="G19" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H19" s="21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="21" t="s">
+        <v>191</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>193</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="G20" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H20" s="21" t="s">
         <v>91</v>
       </c>
     </row>
@@ -2710,22 +3107,22 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>152</v>
+        <v>197</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>153</v>
+        <v>198</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>154</v>
+        <v>199</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>155</v>
+        <v>200</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>156</v>
+        <v>201</v>
       </c>
       <c r="G1" s="14" t="s">
         <v>82</v>
@@ -2733,370 +3130,370 @@
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
-        <v>157</v>
+        <v>202</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>159</v>
+        <v>204</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>160</v>
+        <v>205</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>161</v>
+        <v>206</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>162</v>
+        <v>207</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>164</v>
+        <v>209</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>165</v>
+        <v>210</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>166</v>
+        <v>211</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
-        <v>169</v>
+        <v>214</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>170</v>
+        <v>215</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>171</v>
+        <v>216</v>
       </c>
       <c r="E4" s="22" t="s">
-        <v>172</v>
+        <v>217</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>173</v>
+        <v>218</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>174</v>
+        <v>219</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>175</v>
+        <v>220</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>176</v>
+        <v>221</v>
       </c>
       <c r="F5" s="25" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>177</v>
+        <v>222</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>178</v>
+        <v>223</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>179</v>
+        <v>224</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>180</v>
+        <v>225</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>181</v>
+        <v>226</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>182</v>
+        <v>227</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>183</v>
+        <v>228</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>184</v>
+        <v>229</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>186</v>
+        <v>231</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>187</v>
+        <v>232</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>188</v>
+        <v>233</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>189</v>
+        <v>234</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>190</v>
+        <v>235</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>186</v>
+        <v>231</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>191</v>
+        <v>236</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>192</v>
+        <v>237</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>193</v>
+        <v>238</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>194</v>
+        <v>239</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>196</v>
+        <v>241</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>197</v>
+        <v>242</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>198</v>
+        <v>243</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>162</v>
+        <v>207</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>200</v>
+        <v>245</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>201</v>
+        <v>246</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>202</v>
+        <v>247</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>203</v>
+        <v>248</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>204</v>
+        <v>249</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>205</v>
+        <v>250</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>206</v>
+        <v>251</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>207</v>
+        <v>252</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>208</v>
+        <v>253</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>209</v>
+        <v>254</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>210</v>
+        <v>255</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>211</v>
+        <v>256</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>212</v>
+        <v>257</v>
       </c>
       <c r="D14" s="22" t="s">
+        <v>258</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>259</v>
+      </c>
+      <c r="F14" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="E14" s="22" t="s">
-        <v>214</v>
-      </c>
-      <c r="F14" s="24" t="s">
-        <v>168</v>
-      </c>
       <c r="G14" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>215</v>
+        <v>260</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>216</v>
+        <v>261</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>217</v>
+        <v>262</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>218</v>
+        <v>263</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
-        <v>219</v>
+        <v>264</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>220</v>
+        <v>265</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>221</v>
+        <v>266</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>222</v>
+        <v>267</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
-        <v>223</v>
+        <v>268</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>195</v>
+        <v>240</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>224</v>
+        <v>269</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>225</v>
+        <v>270</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>226</v>
+        <v>271</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -3122,19 +3519,19 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
-        <v>152</v>
+        <v>197</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>227</v>
+        <v>272</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>228</v>
+        <v>273</v>
       </c>
       <c r="D1" s="26" t="s">
-        <v>229</v>
+        <v>274</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>230</v>
+        <v>275</v>
       </c>
       <c r="F1" s="26" t="s">
         <v>82</v>
@@ -3142,122 +3539,122 @@
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
-        <v>231</v>
+        <v>276</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>232</v>
+        <v>277</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>233</v>
+        <v>278</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>234</v>
+        <v>279</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>235</v>
+        <v>280</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>236</v>
+        <v>281</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>237</v>
+        <v>282</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>238</v>
+        <v>283</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>162</v>
+        <v>207</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>239</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
-        <v>240</v>
+        <v>285</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>241</v>
+        <v>286</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>242</v>
+        <v>287</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>243</v>
+        <v>288</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>244</v>
+        <v>289</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>245</v>
+        <v>290</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>246</v>
+        <v>291</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>248</v>
+        <v>293</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>249</v>
+        <v>294</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>250</v>
+        <v>295</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>251</v>
+        <v>296</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>162</v>
+        <v>207</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>252</v>
+        <v>297</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>253</v>
+        <v>298</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>254</v>
+        <v>299</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>255</v>
+        <v>300</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -3282,19 +3679,19 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
-        <v>256</v>
+        <v>301</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>257</v>
+        <v>302</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>258</v>
+        <v>303</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>259</v>
+        <v>304</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>260</v>
+        <v>305</v>
       </c>
       <c r="F1" s="27" t="s">
         <v>82</v>
@@ -3302,182 +3699,182 @@
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
-        <v>261</v>
+        <v>306</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>196</v>
+        <v>241</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>262</v>
+        <v>307</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>263</v>
+        <v>308</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>162</v>
+        <v>207</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>264</v>
+        <v>309</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>265</v>
+        <v>310</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>266</v>
+        <v>311</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>267</v>
+        <v>312</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
-        <v>268</v>
+        <v>313</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>269</v>
+        <v>314</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>270</v>
+        <v>315</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>271</v>
+        <v>316</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>272</v>
+        <v>317</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>273</v>
+        <v>318</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>274</v>
+        <v>319</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>275</v>
+        <v>320</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>276</v>
+        <v>321</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>277</v>
+        <v>322</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>278</v>
+        <v>323</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>279</v>
+        <v>324</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>280</v>
+        <v>325</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>281</v>
+        <v>326</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>282</v>
+        <v>327</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>283</v>
+        <v>328</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>284</v>
+        <v>329</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>285</v>
+        <v>330</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>286</v>
+        <v>331</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>287</v>
+        <v>332</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>288</v>
+        <v>333</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>289</v>
+        <v>334</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>290</v>
+        <v>335</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>291</v>
+        <v>336</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>292</v>
+        <v>337</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>293</v>
+        <v>338</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>294</v>
+        <v>339</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>295</v>
+        <v>340</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -3503,19 +3900,19 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
-        <v>296</v>
+        <v>341</v>
       </c>
       <c r="B1" s="28" t="s">
-        <v>297</v>
+        <v>342</v>
       </c>
       <c r="C1" s="28" t="s">
-        <v>298</v>
+        <v>343</v>
       </c>
       <c r="D1" s="28" t="s">
-        <v>299</v>
+        <v>344</v>
       </c>
       <c r="E1" s="28" t="s">
-        <v>230</v>
+        <v>275</v>
       </c>
       <c r="F1" s="28" t="s">
         <v>82</v>
@@ -3523,122 +3920,122 @@
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
-        <v>300</v>
+        <v>345</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>301</v>
+        <v>346</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>302</v>
+        <v>347</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>303</v>
+        <v>348</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>304</v>
+        <v>349</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>301</v>
+        <v>346</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>305</v>
+        <v>350</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>306</v>
+        <v>351</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
-        <v>307</v>
+        <v>352</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>301</v>
+        <v>346</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>308</v>
+        <v>353</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>309</v>
+        <v>354</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>310</v>
+        <v>355</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>301</v>
+        <v>346</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>311</v>
+        <v>356</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>312</v>
+        <v>357</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>313</v>
+        <v>358</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>315</v>
+        <v>360</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>316</v>
+        <v>361</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>320</v>
+        <v>365</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>163</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -3652,7 +4049,7 @@
   <sheetPr>
     <tabColor rgb="FF64748B"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -3664,33 +4061,33 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
-        <v>321</v>
+        <v>366</v>
       </c>
       <c r="B1" s="29" t="s">
-        <v>322</v>
+        <v>367</v>
       </c>
       <c r="C1" s="29" t="s">
-        <v>323</v>
+        <v>368</v>
       </c>
       <c r="D1" s="29" t="s">
-        <v>324</v>
+        <v>369</v>
       </c>
       <c r="E1" s="29" t="s">
-        <v>325</v>
+        <v>370</v>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
-        <v>326</v>
+        <v>371</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>327</v>
+        <v>372</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>328</v>
+        <v>373</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>329</v>
+        <v>374</v>
       </c>
       <c r="E2" s="23" t="s">
         <v>27</v>
@@ -3698,16 +4095,16 @@
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
-        <v>330</v>
+        <v>375</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>331</v>
+        <v>376</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>332</v>
+        <v>377</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>333</v>
+        <v>378</v>
       </c>
       <c r="E3" s="23" t="s">
         <v>27</v>
@@ -3715,16 +4112,16 @@
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
-        <v>334</v>
+        <v>379</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>335</v>
+        <v>380</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>336</v>
+        <v>381</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>337</v>
+        <v>382</v>
       </c>
       <c r="E4" s="23" t="s">
         <v>27</v>
@@ -3732,16 +4129,16 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="22" t="s">
-        <v>338</v>
+        <v>383</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>339</v>
+        <v>384</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>340</v>
+        <v>385</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>341</v>
+        <v>386</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>27</v>
@@ -3749,16 +4146,16 @@
     </row>
     <row r="6" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
-        <v>342</v>
+        <v>387</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>343</v>
+        <v>388</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>344</v>
+        <v>389</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>345</v>
+        <v>390</v>
       </c>
       <c r="E6" s="23" t="s">
         <v>27</v>
@@ -3766,16 +4163,16 @@
     </row>
     <row r="7" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="22" t="s">
-        <v>346</v>
+        <v>391</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>347</v>
+        <v>392</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>348</v>
+        <v>393</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>349</v>
+        <v>394</v>
       </c>
       <c r="E7" s="23" t="s">
         <v>27</v>
@@ -3783,16 +4180,16 @@
     </row>
     <row r="8" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="22" t="s">
-        <v>350</v>
+        <v>395</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>351</v>
+        <v>396</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>352</v>
+        <v>397</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>353</v>
+        <v>398</v>
       </c>
       <c r="E8" s="23" t="s">
         <v>27</v>
@@ -3800,18 +4197,103 @@
     </row>
     <row r="9" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="22" t="s">
-        <v>354</v>
+        <v>399</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>355</v>
+        <v>400</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>356</v>
+        <v>401</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>357</v>
+        <v>402</v>
       </c>
       <c r="E9" s="23" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="22" t="s">
+        <v>403</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>404</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>405</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>406</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>407</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>408</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>409</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="22" t="s">
+        <v>410</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>411</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>412</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>413</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>414</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>415</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>416</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="22" t="s">
+        <v>417</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>418</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>419</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>420</v>
+      </c>
+      <c r="E14" s="23" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3838,262 +4320,262 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
-        <v>358</v>
+        <v>421</v>
       </c>
       <c r="B1" s="30" t="s">
-        <v>359</v>
+        <v>422</v>
       </c>
       <c r="C1" s="30" t="s">
-        <v>360</v>
+        <v>423</v>
       </c>
       <c r="D1" s="30" t="s">
-        <v>361</v>
+        <v>424</v>
       </c>
       <c r="E1" s="30" t="s">
-        <v>362</v>
+        <v>425</v>
       </c>
       <c r="F1" s="30" t="s">
-        <v>363</v>
+        <v>426</v>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>365</v>
+        <v>428</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>366</v>
+        <v>429</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>367</v>
+        <v>430</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>369</v>
+        <v>432</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>370</v>
+        <v>433</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>371</v>
+        <v>434</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>372</v>
+        <v>435</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>369</v>
+        <v>432</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>373</v>
+        <v>436</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>374</v>
+        <v>437</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>375</v>
+        <v>438</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>369</v>
+        <v>432</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>376</v>
+        <v>439</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>377</v>
+        <v>440</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>372</v>
+        <v>435</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>369</v>
+        <v>432</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>378</v>
+        <v>441</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>379</v>
+        <v>442</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>372</v>
+        <v>435</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>369</v>
+        <v>432</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>380</v>
+        <v>443</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>381</v>
+        <v>444</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>382</v>
+        <v>445</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>369</v>
+        <v>432</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>383</v>
+        <v>446</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>384</v>
+        <v>447</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>385</v>
+        <v>448</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>369</v>
+        <v>432</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>386</v>
+        <v>449</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>387</v>
+        <v>450</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>385</v>
+        <v>448</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>369</v>
+        <v>432</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>388</v>
+        <v>451</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>389</v>
+        <v>452</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>390</v>
+        <v>453</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>369</v>
+        <v>432</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>391</v>
+        <v>454</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>392</v>
+        <v>455</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>385</v>
+        <v>448</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>369</v>
+        <v>432</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>393</v>
+        <v>456</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>394</v>
+        <v>457</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>395</v>
+        <v>458</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>396</v>
+        <v>459</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>397</v>
+        <v>460</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>398</v>
+        <v>461</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>399</v>
+        <v>462</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>400</v>
+        <v>463</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>401</v>
+        <v>464</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>402</v>
+        <v>465</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>403</v>
+        <v>466</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>404</v>
+        <v>467</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add MFA dependencies and harden security
- Install otpauth and qrcode for MFA implementation
- Enforce strict TLS certificate verification in DB connections
- Limit request body size for migration endpoint
- Update audit log query to exclude sensitive fields
</commit_message>
<xml_diff>
--- a/docs/HIPAA_ISO27001_Credentialing_Compliance_Audit_Report.xlsx
+++ b/docs/HIPAA_ISO27001_Credentialing_Compliance_Audit_Report.xlsx
@@ -12,13 +12,14 @@
     <sheet sheetId="6" name="Credentialing_Standards" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="File_By_File_Audit" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="Remediation_Roadmap" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="VLayer_External_Audit_Findings" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="537">
   <si>
     <t>PROFICIO HEALTHCARE CREDENTIALING PLATFORM</t>
   </si>
@@ -29,7 +30,7 @@
     <t>Audit Assessment Date:</t>
   </si>
   <si>
-    <t>2026-09-15 13:21:06 UTC</t>
+    <t>2026-09-17 10:38:42 UTC</t>
   </si>
   <si>
     <t>Audit Scope:</t>
@@ -1422,13 +1423,220 @@
   </si>
   <si>
     <t>SCHEDULED</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Finding Title</t>
+  </si>
+  <si>
+    <t>Source File</t>
+  </si>
+  <si>
+    <t>Line</t>
+  </si>
+  <si>
+    <t>HIPAA Reference CFR</t>
+  </si>
+  <si>
+    <t>Remediation Category</t>
+  </si>
+  <si>
+    <t>Status &amp; Technical Implementation Notes</t>
+  </si>
+  <si>
+    <t>CRITICAL</t>
+  </si>
+  <si>
+    <t>Missing Immediate Access Revocation on User Deletion</t>
+  </si>
+  <si>
+    <t>45 CFR §164.308(a)(3)(ii)(C) - Termination Procedures</t>
+  </si>
+  <si>
+    <t>Hardened &amp; Implemented</t>
+  </si>
+  <si>
+    <t>Implemented mandatory popup requiring delete-user-[userid] with immediate token and session revocation.</t>
+  </si>
+  <si>
+    <t>Encryption issue: TLS certificate validation disabled</t>
+  </si>
+  <si>
+    <t>§164.312(e)(1) - Transmission Security</t>
+  </si>
+  <si>
+    <t>Direct Technical Fix</t>
+  </si>
+  <si>
+    <t>Enforced strict TLS certificate verification (ssl: { rejectUnauthorized: true }).</t>
+  </si>
+  <si>
+    <t>Potential credentials in PostgreSQL connection URI</t>
+  </si>
+  <si>
+    <t>§164.312(a)(1), §164.312(d)</t>
+  </si>
+  <si>
+    <t>Secured connection strings to read strictly from server environment secrets with URI parameter masking.</t>
+  </si>
+  <si>
+    <t>Missing Multi-Factor Authentication for PHI Access</t>
+  </si>
+  <si>
+    <t>45 CFR §164.312(a)(2)(i) - Access Control</t>
+  </si>
+  <si>
+    <t>Feature Addition</t>
+  </si>
+  <si>
+    <t>Requires SMS / TOTP Authenticator 2-Factor challenge on login flow. Pending user consent.</t>
+  </si>
+  <si>
+    <t>Authentication Configuration Without MFA Enabled</t>
+  </si>
+  <si>
+    <t>server/accessRequests.ts</t>
+  </si>
+  <si>
+    <t>NPRM §164.312(d) - Person Authentication</t>
+  </si>
+  <si>
+    <t>MFA requirement on access request and approval endpoints. Pending user consent.</t>
+  </si>
+  <si>
+    <t>Missing Breach Notification Mechanism</t>
+  </si>
+  <si>
+    <t>45 CFR §164.308(a)(6)(ii) - Incident Procedures</t>
+  </si>
+  <si>
+    <t>Requires automated incident reporting &amp; 4-factor risk assessment dashboard. Pending user consent.</t>
+  </si>
+  <si>
+    <t>Requires automated notification dispatch to OCR &amp; affected individuals upon breach. Pending user consent.</t>
+  </si>
+  <si>
+    <t>Missing Immediate Access Revocation</t>
+  </si>
+  <si>
+    <t>Immediate session revocation API hooked into user deletion and role changes.</t>
+  </si>
+  <si>
+    <t>MFA Bypass Detected in Code</t>
+  </si>
+  <si>
+    <t>Remove bypass fallback and mandate verified MFA challenge. Pending user consent.</t>
+  </si>
+  <si>
+    <t>Bulk data deletion operation in seeds/migrations</t>
+  </si>
+  <si>
+    <t>supabase/clean_skeleton_purge.sql</t>
+  </si>
+  <si>
+    <t>§164.530(j) - Retention &amp; Safeguards</t>
+  </si>
+  <si>
+    <t>Guarded migration operations with rollback checks and audit logging.</t>
+  </si>
+  <si>
+    <t>HIGH</t>
+  </si>
+  <si>
+    <t>Encryption issue: Unencrypted HTTP URL in server logs</t>
+  </si>
+  <si>
+    <t>Sanitized server listen logs to remove cleartext http:// protocol prefix.</t>
+  </si>
+  <si>
+    <t>Missing Automatic Session Timeout</t>
+  </si>
+  <si>
+    <t>45 CFR §164.312(a)(2)(iii) - Session Control</t>
+  </si>
+  <si>
+    <t>Enforced 20-minute client inactivity timeout with automatic logout and server token expiry.</t>
+  </si>
+  <si>
+    <t>Authentication Routes Without Rate Limiting</t>
+  </si>
+  <si>
+    <t>45 CFR §164.312(a)(1) - Access Control</t>
+  </si>
+  <si>
+    <t>Added IP sliding-window rate limiters across all authentication and migration routes.</t>
+  </si>
+  <si>
+    <t>Login Flow Without Second Factor Authentication</t>
+  </si>
+  <si>
+    <t>Requires 2FA verification step in login UI. Pending user consent.</t>
+  </si>
+  <si>
+    <t>Missing Vulnerability Scanning Configuration</t>
+  </si>
+  <si>
+    <t>project-level</t>
+  </si>
+  <si>
+    <t>45 CFR §164.308(a)(8) - Evaluation</t>
+  </si>
+  <si>
+    <t>Requires automated in-app vulnerability scanner configuration. Pending user consent.</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>JSON Body Parser Without Size Limit</t>
+  </si>
+  <si>
+    <t>45 CFR §164.308(a)(1)(ii)(D) - System Security</t>
+  </si>
+  <si>
+    <t>Constrained express.json parser explicitly to { limit: "10mb" }.</t>
+  </si>
+  <si>
+    <t>SELECT * on PHI Tables Violates Minimum Necessary</t>
+  </si>
+  <si>
+    <t>45 CFR §164.502(b) - Minimum Necessary</t>
+  </si>
+  <si>
+    <t>Replaced select(*) with explicit minimum necessary non-sensitive columns.</t>
+  </si>
+  <si>
+    <t>Restricted automation queries to explicit credentialing and provider fields.</t>
+  </si>
+  <si>
+    <t>PHI read operation may lack audit logging</t>
+  </si>
+  <si>
+    <t>src/components/reports/ReportsView.tsx</t>
+  </si>
+  <si>
+    <t>§164.312(b) - Audit Controls</t>
+  </si>
+  <si>
+    <t>Integrated logDossierAccess() and centralized audit logging on PHI read views.</t>
+  </si>
+  <si>
+    <t>Web Server Without Security Headers Middleware</t>
+  </si>
+  <si>
+    <t>NPRM Configuration Management</t>
+  </si>
+  <si>
+    <t>Enforced 6 security headers (Strict-Transport-Security, X-Content-Type-Options, CSP, X-Frame-Options).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1501,8 +1709,12 @@
       <color rgb="FF059669"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF2563EB"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1569,6 +1781,16 @@
         <fgColor rgb="FF047857"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF991B1B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE0E7FF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1597,7 +1819,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1680,6 +1902,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4582,4 +4819,509 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FFDC2626"/>
+  </sheetPr>
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="32" t="s">
+        <v>468</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>469</v>
+      </c>
+      <c r="C1" s="32" t="s">
+        <v>470</v>
+      </c>
+      <c r="D1" s="32" t="s">
+        <v>471</v>
+      </c>
+      <c r="E1" s="32" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1" s="32" t="s">
+        <v>473</v>
+      </c>
+      <c r="G1" s="32" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>476</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>410</v>
+      </c>
+      <c r="D2" s="21">
+        <v>799</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>477</v>
+      </c>
+      <c r="F2" s="34" t="s">
+        <v>478</v>
+      </c>
+      <c r="G2" s="22" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>480</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>371</v>
+      </c>
+      <c r="D3" s="21">
+        <v>282</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>481</v>
+      </c>
+      <c r="F3" s="34" t="s">
+        <v>482</v>
+      </c>
+      <c r="G3" s="22" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>484</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>371</v>
+      </c>
+      <c r="D4" s="21">
+        <v>269</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>485</v>
+      </c>
+      <c r="F4" s="34" t="s">
+        <v>482</v>
+      </c>
+      <c r="G4" s="22" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>487</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>403</v>
+      </c>
+      <c r="D5" s="21">
+        <v>19</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>488</v>
+      </c>
+      <c r="F5" s="35" t="s">
+        <v>489</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>491</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>492</v>
+      </c>
+      <c r="D6" s="21">
+        <v>1</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>493</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>489</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>495</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>375</v>
+      </c>
+      <c r="D7" s="21">
+        <v>1382</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>496</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>489</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>495</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>371</v>
+      </c>
+      <c r="D8" s="21">
+        <v>935</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>496</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>489</v>
+      </c>
+      <c r="G8" s="22" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>499</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="D9" s="21">
+        <v>462</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>477</v>
+      </c>
+      <c r="F9" s="34" t="s">
+        <v>478</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>501</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>379</v>
+      </c>
+      <c r="D10" s="21">
+        <v>1014</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>493</v>
+      </c>
+      <c r="F10" s="35" t="s">
+        <v>489</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>503</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>504</v>
+      </c>
+      <c r="D11" s="21">
+        <v>13</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>505</v>
+      </c>
+      <c r="F11" s="34" t="s">
+        <v>482</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="31" t="s">
+        <v>507</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>508</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>371</v>
+      </c>
+      <c r="D12" s="21">
+        <v>1283</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>481</v>
+      </c>
+      <c r="F12" s="34" t="s">
+        <v>482</v>
+      </c>
+      <c r="G12" s="22" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="31" t="s">
+        <v>507</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>510</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>371</v>
+      </c>
+      <c r="D13" s="21">
+        <v>268</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>511</v>
+      </c>
+      <c r="F13" s="34" t="s">
+        <v>478</v>
+      </c>
+      <c r="G13" s="22" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="31" t="s">
+        <v>507</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>513</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>371</v>
+      </c>
+      <c r="D14" s="21">
+        <v>380</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>514</v>
+      </c>
+      <c r="F14" s="34" t="s">
+        <v>482</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="31" t="s">
+        <v>507</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>516</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>399</v>
+      </c>
+      <c r="D15" s="21">
+        <v>121</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>493</v>
+      </c>
+      <c r="F15" s="35" t="s">
+        <v>489</v>
+      </c>
+      <c r="G15" s="22" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="31" t="s">
+        <v>507</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>518</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>519</v>
+      </c>
+      <c r="D16" s="21">
+        <v>1</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>520</v>
+      </c>
+      <c r="F16" s="35" t="s">
+        <v>489</v>
+      </c>
+      <c r="G16" s="22" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="36" t="s">
+        <v>522</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>523</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>371</v>
+      </c>
+      <c r="D17" s="21">
+        <v>261</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>524</v>
+      </c>
+      <c r="F17" s="34" t="s">
+        <v>482</v>
+      </c>
+      <c r="G17" s="22" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="36" t="s">
+        <v>522</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>526</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>371</v>
+      </c>
+      <c r="D18" s="21">
+        <v>1065</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>527</v>
+      </c>
+      <c r="F18" s="34" t="s">
+        <v>482</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="36" t="s">
+        <v>522</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>526</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>417</v>
+      </c>
+      <c r="D19" s="21">
+        <v>264</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>527</v>
+      </c>
+      <c r="F19" s="34" t="s">
+        <v>482</v>
+      </c>
+      <c r="G19" s="22" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="36" t="s">
+        <v>522</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>530</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>531</v>
+      </c>
+      <c r="D20" s="21">
+        <v>125</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>532</v>
+      </c>
+      <c r="F20" s="34" t="s">
+        <v>478</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="36" t="s">
+        <v>522</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>534</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>371</v>
+      </c>
+      <c r="D21" s="21">
+        <v>6</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>535</v>
+      </c>
+      <c r="F21" s="34" t="s">
+        <v>482</v>
+      </c>
+      <c r="G21" s="22" t="s">
+        <v>536</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>